<commit_message>
Fix mechanical and monthly ledger report exports
</commit_message>
<xml_diff>
--- a/backend/app/resources/templates/模板-机械费四页.xlsx
+++ b/backend/app/resources/templates/模板-机械费四页.xlsx
@@ -29,7 +29,7 @@
     <numFmt numFmtId="165" formatCode="0_ "/>
     <numFmt numFmtId="166" formatCode="0.00_);[Red]\(0.00\)"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="17">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -120,8 +120,21 @@
       <color theme="1"/>
       <sz val="10"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Carlito"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Microsoft YaHei"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <name val="Microsoft YaHei"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -140,8 +153,11 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="none"/>
+    </fill>
   </fills>
-  <borders count="14">
+  <borders count="15">
     <border>
       <left/>
       <right/>
@@ -306,11 +322,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -481,6 +506,23 @@
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -847,7 +889,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O7"/>
+  <dimension ref="A1:O11"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="10" defaultRowHeight="21" customHeight="1"/>
   <cols>
     <col width="7.00833333333333" customWidth="1" min="1" max="1"/>
@@ -1050,8 +1092,84 @@
       <c r="N7" s="24" t="n"/>
       <c r="O7" s="24" t="n"/>
     </row>
+    <row r="8" ht="22.5" customHeight="1">
+      <c r="A8" s="71" t="str">
+        <v>注：零租设备含：月份内项目零星外租的各种级别型号规格设备，零租设备使用依据《设备管理程序》7.4.5规定：单台零租设备月度连续租用费用禁止总额接近</v>
+      </c>
+      <c r="B8" s="71"/>
+      <c r="C8" s="71"/>
+      <c r="D8" s="71"/>
+      <c r="E8" s="71"/>
+      <c r="F8" s="71"/>
+      <c r="G8" s="71"/>
+      <c r="H8" s="71"/>
+      <c r="I8" s="71"/>
+      <c r="J8" s="71"/>
+      <c r="K8" s="71"/>
+      <c r="L8" s="71"/>
+      <c r="M8" s="71"/>
+      <c r="N8" s="71"/>
+      <c r="O8" s="71"/>
+    </row>
+    <row r="9" ht="22.5" customHeight="1">
+      <c r="A9" s="69" t="str">
+        <v>         或超过包月租赁价格；包月租赁设备含：连续租用费用总额接近或超过包月租赁价格以上连续租用设备；</v>
+      </c>
+      <c r="B9" s="69"/>
+      <c r="C9" s="69"/>
+      <c r="D9" s="69"/>
+      <c r="E9" s="69"/>
+      <c r="F9" s="69"/>
+      <c r="G9" s="69"/>
+      <c r="H9" s="69"/>
+      <c r="I9" s="69"/>
+      <c r="J9" s="69"/>
+      <c r="K9" s="69"/>
+      <c r="L9" s="69"/>
+      <c r="M9" s="69"/>
+      <c r="N9" s="69"/>
+      <c r="O9" s="69"/>
+    </row>
+    <row r="10" ht="22.5" customHeight="1">
+      <c r="A10" s="69" t="str">
+        <v>     周转性材料依据《物资管理程序》附录二“工程常用材料的大类分项”（七）规定含：片梯、货架、钢方墩、钢丝绳、道木、钢跳板、配电盘（柜）、滚杠、</v>
+      </c>
+      <c r="B10" s="69"/>
+      <c r="C10" s="69"/>
+      <c r="D10" s="69"/>
+      <c r="E10" s="69"/>
+      <c r="F10" s="69"/>
+      <c r="G10" s="69"/>
+      <c r="H10" s="69"/>
+      <c r="I10" s="69"/>
+      <c r="J10" s="69"/>
+      <c r="K10" s="69"/>
+      <c r="L10" s="69"/>
+      <c r="M10" s="69"/>
+      <c r="N10" s="69"/>
+      <c r="O10" s="69"/>
+    </row>
+    <row r="11" ht="22.5" customHeight="1">
+      <c r="A11" s="69" t="str">
+        <v>         临设用35平方（含）以上各种电缆、焊机房、起重抱杆、阀门研磨试压平台、脚手架管、扣件、钢（木）模板、塑料模板、架子车上盘等。</v>
+      </c>
+      <c r="B11" s="69"/>
+      <c r="C11" s="69"/>
+      <c r="D11" s="69"/>
+      <c r="E11" s="69"/>
+      <c r="F11" s="69"/>
+      <c r="G11" s="69"/>
+      <c r="H11" s="69"/>
+      <c r="I11" s="69"/>
+      <c r="J11" s="69"/>
+      <c r="K11" s="69"/>
+      <c r="L11" s="69"/>
+      <c r="M11" s="69"/>
+      <c r="N11" s="69"/>
+      <c r="O11" s="69"/>
+    </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="13">
     <mergeCell ref="J4:N4"/>
     <mergeCell ref="B4:B5"/>
     <mergeCell ref="E4:I4"/>
@@ -1061,6 +1179,10 @@
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="O4:O5"/>
     <mergeCell ref="C4:D4"/>
+    <mergeCell ref="A8:O8"/>
+    <mergeCell ref="A9:O9"/>
+    <mergeCell ref="A10:O10"/>
+    <mergeCell ref="A11:O11"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.4" bottom="0.4" header="0.2" footer="0.2"/>
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>

</xml_diff>